<commit_message>
feat: integrar 52 opiniões em 7 grupos na análise dos preâmbulos
- Expandir OPINIAO_DADOS de 18 para 52 organizações (4-tuple com campo grupo)
- Actualizar gerar_tabela_opiniao(): subheadings por grupo + filtro dropdown JS
- Actualizar gerar_excel() Sec4: coluna Grupo, separador por grupo, cores pastel por grupo
- Actualizar gerar_word() Sec4: tabela condensada 3-col (org + grupo + síntese posições)
- Actualizar hero tags: "18 pareceres" → "52 pareceres (7 grupos)"
- Regenerar HTML, Word e Excel

https://claude.ai/code/session_013gc37ZfszD9QAJQ5M1gWcB
</commit_message>
<xml_diff>
--- a/analise_preambulos_opinoes.xlsx
+++ b/analise_preambulos_opinoes.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,7 +62,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="002D4059"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00666666"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -79,7 +90,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +129,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EAF4EA"/>
+        <bgColor rgb="00EAF4EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAD6D6"/>
+        <bgColor rgb="00EAD6D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F5E7D1"/>
         <bgColor rgb="00F5E7D1"/>
       </patternFill>
@@ -130,8 +153,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAD6D6"/>
-        <bgColor rgb="00EAD6D6"/>
+        <fgColor rgb="00EAF0FA"/>
+        <bgColor rgb="00EAF0FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8EA"/>
+        <bgColor rgb="00FFF8EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF0EA"/>
+        <bgColor rgb="00FFF0EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5EAFA"/>
+        <bgColor rgb="00F5EAFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF7FA"/>
+        <bgColor rgb="00EAF7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0EAF5"/>
+        <bgColor rgb="00F0EAF5"/>
       </patternFill>
     </fill>
     <fill>
@@ -167,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -187,46 +240,85 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1095,26 +1187,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Matriz de Opiniões: 18 Organizações × 10 Temas</t>
+          <t>Matriz de Opiniões: 52 Organizações × 10 Temas (7 grupos)</t>
         </is>
       </c>
     </row>
@@ -1124,554 +1217,2281 @@
           <t>Organização</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Limiar Art. 4</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Proibição venda lojas</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Castração cirúrgica</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>Coleiras elétricas</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Cães de caça</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>Rastreabi- lidade</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Braquice- fálicos</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>Acorren- tamento</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>Animais errantes</t>
         </is>
       </c>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
         <is>
           <t>Venda online</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
         <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Eurogroup for Animals</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr"/>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L5" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>LAV Onlus</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr"/>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L6" s="14" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
           <t>AWI / Ecuavet</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="10" t="inlineStr"/>
-      <c r="D4" s="10" t="inlineStr"/>
-      <c r="E4" s="10" t="inlineStr"/>
-      <c r="F4" s="10" t="inlineStr"/>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr"/>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição total</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr"/>
-      <c r="K4" s="10" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr"/>
+      <c r="E7" s="14" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr"/>
+      <c r="G7" s="14" t="inlineStr"/>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="inlineStr"/>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr"/>
+      <c r="L7" s="14" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>AnimaNaturalis</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="10" t="inlineStr"/>
-      <c r="D5" s="10" t="inlineStr"/>
-      <c r="E5" s="10" t="inlineStr"/>
-      <c r="F5" s="10" t="inlineStr"/>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr"/>
-      <c r="I5" s="10" t="inlineStr"/>
-      <c r="J5" s="10" t="inlineStr"/>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>FACE</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>△ revisão</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr"/>
-      <c r="D6" s="10" t="inlineStr"/>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>△ uso regulado</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>△ derrogação</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr"/>
-      <c r="H6" s="10" t="inlineStr"/>
-      <c r="I6" s="10" t="inlineStr"/>
-      <c r="J6" s="10" t="inlineStr"/>
-      <c r="K6" s="10" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr"/>
+      <c r="D8" s="14" t="inlineStr"/>
+      <c r="E8" s="14" t="inlineStr"/>
+      <c r="F8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr"/>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr"/>
+      <c r="J8" s="14" t="inlineStr"/>
+      <c r="K8" s="14" t="inlineStr"/>
+      <c r="L8" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>VETO</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr"/>
+      <c r="D9" s="14" t="inlineStr"/>
+      <c r="E9" s="14" t="inlineStr"/>
+      <c r="F9" s="14" t="inlineStr"/>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr"/>
+      <c r="J9" s="14" t="inlineStr"/>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L9" s="14" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>SEY Animal Welfare Finland</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr"/>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr"/>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr"/>
+      <c r="J10" s="14" t="inlineStr"/>
+      <c r="K10" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Norwegian Society for Protection</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr"/>
+      <c r="E11" s="14" t="inlineStr"/>
+      <c r="F11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr"/>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I11" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="inlineStr"/>
+      <c r="K11" s="14" t="inlineStr"/>
+      <c r="L11" s="14" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Tierschutz-LASA</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
+      <c r="E12" s="14" t="inlineStr"/>
+      <c r="F12" s="14" t="inlineStr"/>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr"/>
+      <c r="I12" s="14" t="inlineStr"/>
+      <c r="J12" s="14" t="inlineStr"/>
+      <c r="K12" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L12" s="14" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>EUCED</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr"/>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr"/>
+      <c r="G13" s="14" t="inlineStr"/>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="inlineStr"/>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Animal Protection Denmark</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr"/>
+      <c r="G14" s="14" t="inlineStr"/>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I14" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="K14" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Djurskyddet Sverige</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Finnish Centre for Animal Welfare</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr"/>
+      <c r="E16" s="14" t="inlineStr"/>
+      <c r="F16" s="14" t="inlineStr"/>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr"/>
+      <c r="L16" s="14" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Dutch Assoc. Protection Animals</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr"/>
+      <c r="E17" s="14" t="inlineStr"/>
+      <c r="F17" s="14" t="inlineStr"/>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr"/>
+      <c r="K17" s="14" t="inlineStr"/>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>EU Dog &amp; Cat Alliance</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr"/>
+      <c r="F18" s="14" t="inlineStr"/>
+      <c r="G18" s="14" t="inlineStr"/>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="inlineStr"/>
+      <c r="K18" s="14" t="inlineStr"/>
+      <c r="L18" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Brigitte Bardot Foundation</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="inlineStr"/>
+      <c r="K19" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>PETA Deutschland</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I20" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J20" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>NOAH – for dyrs rettigheter</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>SOS Galgos</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F22" s="14" t="inlineStr"/>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L22" s="14" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>FENPCA</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F23" s="14" t="inlineStr"/>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I23" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J23" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L23" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>LAU KATU ELKARTEA</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F24" s="14" t="inlineStr"/>
+      <c r="G24" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="inlineStr"/>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Asociación HAIEKIN</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr"/>
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J25" s="14" t="inlineStr"/>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>APARIOJA (La Rioja)</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr"/>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I26" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J26" s="14" t="inlineStr"/>
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>MIS AMIGAS LAS PALOMAS</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr"/>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I27" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J27" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="K27" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L27" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>INTERcids</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Bem-estar animal</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr"/>
+      <c r="D28" s="14" t="inlineStr"/>
+      <c r="E28" s="14" t="inlineStr"/>
+      <c r="F28" s="14" t="inlineStr"/>
+      <c r="G28" s="14" t="inlineStr"/>
+      <c r="H28" s="14" t="inlineStr"/>
+      <c r="I28" s="14" t="inlineStr"/>
+      <c r="J28" s="14" t="inlineStr"/>
+      <c r="K28" s="14" t="inlineStr"/>
+      <c r="L28" s="14" t="inlineStr"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>FVE (Fed. Veterinários EU)</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr"/>
+      <c r="G30" s="14" t="inlineStr"/>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J30" s="14" t="inlineStr"/>
+      <c r="K30" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L30" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>WSAVA</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr"/>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr"/>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I31" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="K31" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Danish Veterinary Assoc.</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr"/>
+      <c r="G32" s="14" t="inlineStr"/>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I32" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J32" s="14" t="inlineStr"/>
+      <c r="K32" s="14" t="inlineStr"/>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="inlineStr">
+        <is>
+          <t>Federal Chamber Vet. (BTK 🇩🇪)</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr"/>
+      <c r="E33" s="14" t="inlineStr"/>
+      <c r="F33" s="14" t="inlineStr"/>
+      <c r="G33" s="14" t="inlineStr"/>
+      <c r="H33" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I33" s="14" t="inlineStr"/>
+      <c r="J33" s="14" t="inlineStr"/>
+      <c r="K33" s="14" t="inlineStr"/>
+      <c r="L33" s="14" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Norwegian Vet. Nurses Assoc.</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr"/>
+      <c r="D34" s="14" t="inlineStr"/>
+      <c r="E34" s="14" t="inlineStr"/>
+      <c r="F34" s="14" t="inlineStr"/>
+      <c r="G34" s="14" t="inlineStr"/>
+      <c r="H34" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I34" s="14" t="inlineStr"/>
+      <c r="J34" s="14" t="inlineStr"/>
+      <c r="K34" s="14" t="inlineStr"/>
+      <c r="L34" s="14" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
+        <is>
+          <t>Manteca / UAB</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr"/>
+      <c r="D35" s="14" t="inlineStr"/>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr"/>
+      <c r="G35" s="14" t="inlineStr"/>
+      <c r="H35" s="14" t="inlineStr"/>
+      <c r="I35" s="14" t="inlineStr"/>
+      <c r="J35" s="14" t="inlineStr"/>
+      <c r="K35" s="14" t="inlineStr"/>
+      <c r="L35" s="14" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
+        <is>
+          <t>UAB (Comportamento animal)</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr"/>
+      <c r="D36" s="14" t="inlineStr"/>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="inlineStr"/>
+      <c r="G36" s="14" t="inlineStr"/>
+      <c r="H36" s="14" t="inlineStr"/>
+      <c r="I36" s="14" t="inlineStr"/>
+      <c r="J36" s="14" t="inlineStr"/>
+      <c r="K36" s="14" t="inlineStr"/>
+      <c r="L36" s="14" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>VIRBAC</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>Veterinária</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr"/>
+      <c r="D37" s="14" t="inlineStr"/>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="F37" s="14" t="inlineStr"/>
+      <c r="G37" s="14" t="inlineStr"/>
+      <c r="H37" s="14" t="inlineStr"/>
+      <c r="I37" s="14" t="inlineStr"/>
+      <c r="J37" s="14" t="inlineStr"/>
+      <c r="K37" s="14" t="inlineStr"/>
+      <c r="L37" s="14" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>Kennel clubs e felinologia</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="21" t="inlineStr">
         <is>
           <t>Koninklijke Hondenbescherming</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr"/>
-      <c r="E7" s="10" t="inlineStr"/>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr"/>
-      <c r="J7" s="10" t="inlineStr"/>
-      <c r="K7" s="10" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Manteca / UAB</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="10" t="inlineStr"/>
-      <c r="D8" s="10" t="inlineStr">
-        <is>
-          <t>✖ crítica</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="inlineStr"/>
-      <c r="F8" s="10" t="inlineStr"/>
-      <c r="G8" s="10" t="inlineStr"/>
-      <c r="H8" s="10" t="inlineStr"/>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>Kennel clubs e felinologia</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr"/>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="inlineStr"/>
+      <c r="F39" s="14" t="inlineStr"/>
+      <c r="G39" s="14" t="inlineStr"/>
+      <c r="H39" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I39" s="14" t="inlineStr"/>
+      <c r="J39" s="14" t="inlineStr"/>
+      <c r="K39" s="14" t="inlineStr"/>
+      <c r="L39" s="14" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="21" t="inlineStr">
+        <is>
+          <t>The Dutch Kennel Club</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>Kennel clubs e felinologia</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr"/>
+      <c r="E40" s="14" t="inlineStr"/>
+      <c r="F40" s="14" t="inlineStr"/>
+      <c r="G40" s="14" t="inlineStr"/>
+      <c r="H40" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I40" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="inlineStr"/>
+      <c r="K40" s="14" t="inlineStr"/>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t>Norwegian Kennel Club</t>
+        </is>
+      </c>
+      <c r="B41" s="22" t="inlineStr">
+        <is>
+          <t>Kennel clubs e felinologia</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="F41" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="G41" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I41" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J41" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="K41" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L41" s="14" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>Lithuanian Felinology (Bubaste)</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>Kennel clubs e felinologia</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr"/>
+      <c r="D42" s="14" t="inlineStr"/>
+      <c r="E42" s="14" t="inlineStr"/>
+      <c r="F42" s="14" t="inlineStr"/>
+      <c r="G42" s="14" t="inlineStr"/>
+      <c r="H42" s="14" t="inlineStr"/>
+      <c r="I42" s="14" t="inlineStr"/>
+      <c r="J42" s="14" t="inlineStr"/>
+      <c r="K42" s="14" t="inlineStr"/>
+      <c r="L42" s="14" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>Caçadores e uso funcional</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="24" t="inlineStr">
+        <is>
+          <t>FACE (Fed. Caçadores EU)</t>
+        </is>
+      </c>
+      <c r="B44" s="25" t="inlineStr">
+        <is>
+          <t>Caçadores e uso funcional</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr"/>
+      <c r="E44" s="14" t="inlineStr"/>
+      <c r="F44" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="G44" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H44" s="14" t="inlineStr"/>
+      <c r="I44" s="14" t="inlineStr"/>
+      <c r="J44" s="14" t="inlineStr"/>
+      <c r="K44" s="14" t="inlineStr"/>
+      <c r="L44" s="14" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="24" t="inlineStr">
+        <is>
+          <t>Féd. Nationale Chasseurs (FR)</t>
+        </is>
+      </c>
+      <c r="B45" s="25" t="inlineStr">
+        <is>
+          <t>Caçadores e uso funcional</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr"/>
+      <c r="E45" s="14" t="inlineStr"/>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="G45" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H45" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr"/>
+      <c r="J45" s="14" t="inlineStr"/>
+      <c r="K45" s="14" t="inlineStr"/>
+      <c r="L45" s="14" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="inlineStr">
+        <is>
+          <t>Real Fed. Española de Caza</t>
+        </is>
+      </c>
+      <c r="B46" s="25" t="inlineStr">
+        <is>
+          <t>Caçadores e uso funcional</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr"/>
+      <c r="E46" s="14" t="inlineStr"/>
+      <c r="F46" s="14" t="inlineStr"/>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="H46" s="14" t="inlineStr"/>
+      <c r="I46" s="14" t="inlineStr"/>
+      <c r="J46" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="K46" s="14" t="inlineStr"/>
+      <c r="L46" s="14" t="inlineStr"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>FEDIAF</t>
+        </is>
+      </c>
+      <c r="B48" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C48" s="14" t="inlineStr"/>
+      <c r="D48" s="14" t="inlineStr"/>
+      <c r="E48" s="14" t="inlineStr"/>
+      <c r="F48" s="14" t="inlineStr"/>
+      <c r="G48" s="14" t="inlineStr"/>
+      <c r="H48" s="14" t="inlineStr"/>
+      <c r="I48" s="14" t="inlineStr"/>
+      <c r="J48" s="14" t="inlineStr"/>
+      <c r="K48" s="14" t="inlineStr"/>
+      <c r="L48" s="14" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
         <is>
           <t>MSD Animal Health</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="10" t="inlineStr"/>
-      <c r="E9" s="10" t="inlineStr"/>
-      <c r="F9" s="10" t="inlineStr"/>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>✔ reforço</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr"/>
-      <c r="I9" s="10" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Norwegian Society</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>△ limiar ↓</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr"/>
-      <c r="D10" s="10" t="inlineStr"/>
-      <c r="E10" s="10" t="inlineStr"/>
-      <c r="F10" s="10" t="inlineStr"/>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>⚠ COI</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr"/>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>SEY Animal Welfare Finland</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr"/>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição total</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr"/>
-      <c r="G11" s="10" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr"/>
-      <c r="I11" s="10" t="inlineStr"/>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="K11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>VETO</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="10" t="inlineStr"/>
-      <c r="D12" s="10" t="inlineStr"/>
-      <c r="E12" s="10" t="inlineStr"/>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>✖ anti-derrg.</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr"/>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>⚠ galgos</t>
-        </is>
-      </c>
-      <c r="K12" s="10" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>VIRBAC</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>✖ crítica</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="inlineStr"/>
-      <c r="F13" s="10" t="inlineStr"/>
-      <c r="G13" s="10" t="inlineStr"/>
-      <c r="H13" s="10" t="inlineStr"/>
-      <c r="I13" s="10" t="inlineStr"/>
-      <c r="J13" s="10" t="inlineStr"/>
-      <c r="K13" s="10" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>UAB Comportamental</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="10" t="inlineStr"/>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>✖ crítica</t>
-        </is>
-      </c>
-      <c r="E14" s="10" t="inlineStr"/>
-      <c r="F14" s="10" t="inlineStr"/>
-      <c r="G14" s="10" t="inlineStr"/>
-      <c r="H14" s="10" t="inlineStr"/>
-      <c r="I14" s="10" t="inlineStr"/>
-      <c r="J14" s="10" t="inlineStr"/>
-      <c r="K14" s="10" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Féd. nationale chasseurs (FR)</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>△ revisão</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr"/>
-      <c r="D15" s="10" t="inlineStr"/>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>△ uso regulado</t>
-        </is>
-      </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>△ derrogação</t>
-        </is>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>△ flexibil.</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr"/>
-      <c r="I15" s="10" t="inlineStr"/>
-      <c r="J15" s="10" t="inlineStr"/>
-      <c r="K15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Tierschutz-LASA</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr"/>
-      <c r="C16" s="10" t="inlineStr"/>
-      <c r="D16" s="10" t="inlineStr"/>
-      <c r="E16" s="10" t="inlineStr"/>
-      <c r="F16" s="10" t="inlineStr">
-        <is>
-          <t>✖ anti-derrg.</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr"/>
-      <c r="H16" s="10" t="inlineStr"/>
-      <c r="I16" s="10" t="inlineStr"/>
-      <c r="J16" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="K16" s="10" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>EUCED</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr"/>
-      <c r="C17" s="10" t="inlineStr"/>
-      <c r="D17" s="10" t="inlineStr"/>
-      <c r="E17" s="10" t="inlineStr"/>
-      <c r="F17" s="10" t="inlineStr"/>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr"/>
-      <c r="I17" s="10" t="inlineStr"/>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>FEDIAF</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr"/>
-      <c r="C18" s="10" t="inlineStr"/>
-      <c r="D18" s="10" t="inlineStr"/>
-      <c r="E18" s="10" t="inlineStr"/>
-      <c r="F18" s="10" t="inlineStr"/>
-      <c r="G18" s="10" t="inlineStr"/>
-      <c r="H18" s="10" t="inlineStr"/>
-      <c r="I18" s="10" t="inlineStr"/>
-      <c r="J18" s="10" t="inlineStr"/>
-      <c r="K18" s="10" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Eurogroup for Animals</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>✖ suprimir isenções</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr"/>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição total</t>
-        </is>
-      </c>
-      <c r="F19" s="10" t="inlineStr"/>
-      <c r="G19" s="10" t="inlineStr">
-        <is>
-          <t>✔ universal</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibir criação</t>
-        </is>
-      </c>
-      <c r="I19" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição total</t>
-        </is>
-      </c>
-      <c r="J19" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="B49" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr"/>
+      <c r="D49" s="14" t="inlineStr"/>
+      <c r="E49" s="14" t="inlineStr"/>
+      <c r="F49" s="14" t="inlineStr"/>
+      <c r="G49" s="14" t="inlineStr"/>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="I49" s="14" t="inlineStr"/>
+      <c r="J49" s="14" t="inlineStr"/>
+      <c r="K49" s="14" t="inlineStr"/>
+      <c r="L49" s="14" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>AnimalhealthEurope</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr"/>
+      <c r="F50" s="14" t="inlineStr"/>
+      <c r="G50" s="14" t="inlineStr"/>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I50" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J50" s="14" t="inlineStr"/>
+      <c r="K50" s="14" t="inlineStr"/>
+      <c r="L50" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>Electronic Collar Manufacturers</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr"/>
+      <c r="D51" s="14" t="inlineStr"/>
+      <c r="E51" s="14" t="inlineStr"/>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="H51" s="14" t="inlineStr"/>
+      <c r="I51" s="14" t="inlineStr"/>
+      <c r="J51" s="14" t="inlineStr"/>
+      <c r="K51" s="14" t="inlineStr"/>
+      <c r="L51" s="14" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>Assoc. Responsible Dog Owners</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr"/>
+      <c r="D52" s="14" t="inlineStr"/>
+      <c r="E52" s="14" t="inlineStr"/>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="G52" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H52" s="14" t="inlineStr"/>
+      <c r="I52" s="14" t="inlineStr"/>
+      <c r="J52" s="14" t="inlineStr"/>
+      <c r="K52" s="14" t="inlineStr"/>
+      <c r="L52" s="14" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>Classifieds Marketplaces Europe</t>
+        </is>
+      </c>
+      <c r="B53" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr"/>
+      <c r="D53" s="14" t="inlineStr"/>
+      <c r="E53" s="14" t="inlineStr"/>
+      <c r="F53" s="14" t="inlineStr"/>
+      <c r="G53" s="14" t="inlineStr"/>
+      <c r="H53" s="14" t="inlineStr"/>
+      <c r="I53" s="14" t="inlineStr"/>
+      <c r="J53" s="14" t="inlineStr"/>
+      <c r="K53" s="14" t="inlineStr"/>
+      <c r="L53" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="27" t="inlineStr">
+        <is>
+          <t>European Pet Organization (EPO)</t>
+        </is>
+      </c>
+      <c r="B54" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr"/>
+      <c r="D54" s="14" t="inlineStr"/>
+      <c r="E54" s="14" t="inlineStr"/>
+      <c r="F54" s="14" t="inlineStr"/>
+      <c r="G54" s="14" t="inlineStr"/>
+      <c r="H54" s="14" t="inlineStr"/>
+      <c r="I54" s="14" t="inlineStr"/>
+      <c r="J54" s="14" t="inlineStr"/>
+      <c r="K54" s="14" t="inlineStr"/>
+      <c r="L54" s="14" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="27" t="inlineStr">
         <is>
           <t>World Dog Alliance</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr"/>
-      <c r="C20" s="10" t="inlineStr"/>
-      <c r="D20" s="10" t="inlineStr"/>
-      <c r="E20" s="10" t="inlineStr"/>
-      <c r="F20" s="10" t="inlineStr"/>
-      <c r="G20" s="10" t="inlineStr"/>
-      <c r="H20" s="10" t="inlineStr"/>
-      <c r="I20" s="10" t="inlineStr"/>
-      <c r="J20" s="10" t="inlineStr"/>
-      <c r="K20" s="10" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>LAV Onlus</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>✖ suprimir isenções</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr"/>
-      <c r="E21" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição total</t>
-        </is>
-      </c>
-      <c r="F21" s="10" t="inlineStr"/>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>✔ universal</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibir criação</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>✖ proibição total</t>
-        </is>
-      </c>
-      <c r="J21" s="11" t="inlineStr">
-        <is>
-          <t>⚠</t>
-        </is>
-      </c>
-      <c r="K21" s="10" t="inlineStr"/>
+      <c r="B55" s="28" t="inlineStr">
+        <is>
+          <t>Indústria e comércio</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr"/>
+      <c r="D55" s="14" t="inlineStr"/>
+      <c r="E55" s="14" t="inlineStr"/>
+      <c r="F55" s="14" t="inlineStr"/>
+      <c r="G55" s="14" t="inlineStr"/>
+      <c r="H55" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I55" s="14" t="inlineStr"/>
+      <c r="J55" s="14" t="inlineStr"/>
+      <c r="K55" s="14" t="inlineStr"/>
+      <c r="L55" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="29" t="inlineStr">
+        <is>
+          <t>Rastreabilidade e I&amp;R</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="30" t="inlineStr">
+        <is>
+          <t>EuroPetNet</t>
+        </is>
+      </c>
+      <c r="B57" s="31" t="inlineStr">
+        <is>
+          <t>Rastreabilidade e I&amp;R</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr"/>
+      <c r="D57" s="14" t="inlineStr"/>
+      <c r="E57" s="14" t="inlineStr"/>
+      <c r="F57" s="14" t="inlineStr"/>
+      <c r="G57" s="14" t="inlineStr"/>
+      <c r="H57" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I57" s="14" t="inlineStr"/>
+      <c r="J57" s="14" t="inlineStr"/>
+      <c r="K57" s="14" t="inlineStr"/>
+      <c r="L57" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="30" t="inlineStr">
+        <is>
+          <t>K&amp;R Network</t>
+        </is>
+      </c>
+      <c r="B58" s="31" t="inlineStr">
+        <is>
+          <t>Rastreabilidade e I&amp;R</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr"/>
+      <c r="E58" s="14" t="inlineStr"/>
+      <c r="F58" s="14" t="inlineStr"/>
+      <c r="G58" s="14" t="inlineStr"/>
+      <c r="H58" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I58" s="14" t="inlineStr"/>
+      <c r="J58" s="14" t="inlineStr"/>
+      <c r="K58" s="14" t="inlineStr"/>
+      <c r="L58" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="30" t="inlineStr">
+        <is>
+          <t>TASSO e.V.</t>
+        </is>
+      </c>
+      <c r="B59" s="31" t="inlineStr">
+        <is>
+          <t>Rastreabilidade e I&amp;R</t>
+        </is>
+      </c>
+      <c r="C59" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr"/>
+      <c r="E59" s="14" t="inlineStr"/>
+      <c r="F59" s="14" t="inlineStr"/>
+      <c r="G59" s="14" t="inlineStr"/>
+      <c r="H59" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I59" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J59" s="14" t="inlineStr"/>
+      <c r="K59" s="14" t="inlineStr"/>
+      <c r="L59" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="32" t="inlineStr">
+        <is>
+          <t>Autoridades públicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="33" t="inlineStr">
+        <is>
+          <t>Bundesministerium (🇩🇪)</t>
+        </is>
+      </c>
+      <c r="B61" s="34" t="inlineStr">
+        <is>
+          <t>Autoridades públicas</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr"/>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F61" s="14" t="inlineStr"/>
+      <c r="G61" s="14" t="inlineStr"/>
+      <c r="H61" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I61" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J61" s="14" t="inlineStr"/>
+      <c r="K61" s="14" t="inlineStr"/>
+      <c r="L61" s="14" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="33" t="inlineStr">
+        <is>
+          <t>Czech National Authority</t>
+        </is>
+      </c>
+      <c r="B62" s="34" t="inlineStr">
+        <is>
+          <t>Autoridades públicas</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>Contra</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="F62" s="14" t="inlineStr"/>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="H62" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I62" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J62" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="K62" s="14" t="inlineStr"/>
+      <c r="L62" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="33" t="inlineStr">
+        <is>
+          <t>Norwegian Food Safety Auth.</t>
+        </is>
+      </c>
+      <c r="B63" s="34" t="inlineStr">
+        <is>
+          <t>Autoridades públicas</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="D63" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="E63" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="G63" s="16" t="inlineStr">
+        <is>
+          <t>Derrogação</t>
+        </is>
+      </c>
+      <c r="H63" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="I63" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="J63" s="15" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="K63" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+      <c r="L63" s="13" t="inlineStr">
+        <is>
+          <t>Favor</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="33" t="inlineStr">
+        <is>
+          <t>Fundación Vet+i (🇪🇸)</t>
+        </is>
+      </c>
+      <c r="B64" s="34" t="inlineStr">
+        <is>
+          <t>Autoridades públicas</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr"/>
+      <c r="D64" s="14" t="inlineStr"/>
+      <c r="E64" s="14" t="inlineStr"/>
+      <c r="F64" s="14" t="inlineStr"/>
+      <c r="G64" s="14" t="inlineStr"/>
+      <c r="H64" s="14" t="inlineStr"/>
+      <c r="I64" s="14" t="inlineStr"/>
+      <c r="J64" s="14" t="inlineStr"/>
+      <c r="K64" s="14" t="inlineStr"/>
+      <c r="L64" s="14" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
+    <mergeCell ref="A38:L38"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A47:L47"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A56:L56"/>
+    <mergeCell ref="A4:L4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1699,22 +3519,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="35" t="inlineStr">
         <is>
           <t>Tema</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="35" t="inlineStr">
         <is>
           <t>Polémica</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="35" t="inlineStr">
         <is>
           <t>Impacto PT</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="35" t="inlineStr">
         <is>
           <t>Nota específica</t>
         </is>
@@ -1950,24 +3770,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>Animais registados (SIAC, outubro 2023)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -2059,24 +3879,24 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>Animais errantes (Censo ICNF / Univ. Aveiro, 2023)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -2168,24 +3988,24 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="36" t="inlineStr">
         <is>
           <t>Abandono (dados 2022)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -2277,24 +4097,24 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="36" t="inlineStr">
         <is>
           <t>Contexto comparativo europeu</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
@@ -2393,67 +4213,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="37" t="inlineStr">
         <is>
           <t>Paleta de cores — Legenda</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>Verde pastel</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="39" t="inlineStr">
         <is>
           <t>Posição Favor / Apoio nas opiniões</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="40" t="inlineStr">
         <is>
           <t>Rosa suave</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>Posição Contra / Crítica nas opiniões</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>Bege suave</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="39" t="inlineStr">
         <is>
           <t>Propõe reforço / Crítica moderada</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t>Roxo pastel</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="39" t="inlineStr">
         <is>
           <t>Propõe derrogação / Flexibilização</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Cinzento suave</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="39" t="inlineStr">
         <is>
           <t>Impacto Muito Alto em Portugal</t>
         </is>

</xml_diff>